<commit_message>
SPPBJ KAK: hilangkan tabel point B, jadikan list polos sesuai lampiran
- Template: hapus merge header 71-72 (point 2 tak lagi ketelan),
  deborder kolom A-D rows 71-90 (A->s116, D->s117 wrap, B/C->s121),
  rows 71-76 auto-height supaya teks wrap penuh
- fill.ts: nomor point ditulis "1." (string) cocok format lampiran

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/sppbj/sppbj.xlsx
+++ b/templates/sppbj/sppbj.xlsx
@@ -14147,88 +14147,88 @@
       </c>
       <c r="G70" s="121"/>
     </row>
-    <row r="71" ht="14.25" customHeight="1">
-      <c r="A71" s="50" t="s">
+    <row r="71">
+      <c r="A71" s="116" t="s">
         <v>468</v>
       </c>
-      <c r="B71" s="50" t="s">
+      <c r="B71" s="121" t="s">
         <v>469</v>
       </c>
-      <c r="C71" s="50" t="s">
+      <c r="C71" s="121" t="s">
         <v>470</v>
       </c>
-      <c r="D71" s="50" t="s">
+      <c r="D71" s="117" t="s">
         <v>471</v>
       </c>
       <c r="E71" s="121"/>
       <c r="F71" s="121"/>
       <c r="G71" s="121"/>
     </row>
-    <row r="72" ht="14.25" customHeight="1">
-      <c r="A72" s="53"/>
-      <c r="B72" s="53"/>
-      <c r="C72" s="53"/>
-      <c r="D72" s="53"/>
+    <row r="72">
+      <c r="A72" s="116"/>
+      <c r="B72" s="121"/>
+      <c r="C72" s="121"/>
+      <c r="D72" s="117"/>
       <c r="E72" s="121"/>
       <c r="F72" s="121"/>
       <c r="G72" s="121"/>
     </row>
-    <row r="73" ht="14.25" customHeight="1">
-      <c r="A73" s="55"/>
-      <c r="B73" s="56"/>
-      <c r="C73" s="56"/>
-      <c r="D73" s="57" t="s">
+    <row r="73">
+      <c r="A73" s="116"/>
+      <c r="B73" s="121"/>
+      <c r="C73" s="121"/>
+      <c r="D73" s="117" t="s">
         <v>58</v>
       </c>
       <c r="E73" s="121"/>
       <c r="F73" s="121"/>
       <c r="G73" s="121"/>
     </row>
-    <row r="74" ht="14.25" customHeight="1">
-      <c r="A74" s="55">
+    <row r="74">
+      <c r="A74" s="116">
         <v>1.0</v>
       </c>
-      <c r="B74" s="56">
+      <c r="B74" s="121">
         <v>1.0</v>
       </c>
-      <c r="C74" s="56" t="s">
+      <c r="C74" s="121" t="s">
         <v>475</v>
       </c>
-      <c r="D74" s="61" t="s">
+      <c r="D74" s="117" t="s">
         <v>476</v>
       </c>
       <c r="E74" s="121"/>
       <c r="F74" s="121"/>
       <c r="G74" s="121"/>
     </row>
-    <row r="75" ht="14.25" customHeight="1">
-      <c r="A75" s="55">
+    <row r="75">
+      <c r="A75" s="116">
         <v>2.0</v>
       </c>
-      <c r="B75" s="56">
+      <c r="B75" s="121">
         <v>7.0</v>
       </c>
-      <c r="C75" s="56" t="s">
+      <c r="C75" s="121" t="s">
         <v>477</v>
       </c>
-      <c r="D75" s="61" t="s">
+      <c r="D75" s="117" t="s">
         <v>478</v>
       </c>
       <c r="E75" s="121"/>
       <c r="F75" s="121"/>
       <c r="G75" s="121"/>
     </row>
-    <row r="76" ht="14.25" customHeight="1">
-      <c r="A76" s="55">
+    <row r="76">
+      <c r="A76" s="116">
         <v>3.0</v>
       </c>
-      <c r="B76" s="56">
+      <c r="B76" s="121">
         <v>18.0</v>
       </c>
-      <c r="C76" s="56" t="s">
+      <c r="C76" s="121" t="s">
         <v>475</v>
       </c>
-      <c r="D76" s="61" t="s">
+      <c r="D76" s="117" t="s">
         <v>479</v>
       </c>
       <c r="E76" s="121"/>
@@ -14236,16 +14236,16 @@
       <c r="G76" s="121"/>
     </row>
     <row r="77" ht="14.25" customHeight="1">
-      <c r="A77" s="55">
+      <c r="A77" s="116">
         <v>4.0</v>
       </c>
-      <c r="B77" s="56">
+      <c r="B77" s="121">
         <v>9.0</v>
       </c>
-      <c r="C77" s="56" t="s">
+      <c r="C77" s="121" t="s">
         <v>475</v>
       </c>
-      <c r="D77" s="61" t="s">
+      <c r="D77" s="117" t="s">
         <v>480</v>
       </c>
       <c r="E77" s="121"/>
@@ -14253,16 +14253,16 @@
       <c r="G77" s="121"/>
     </row>
     <row r="78" ht="14.25" customHeight="1">
-      <c r="A78" s="55">
+      <c r="A78" s="116">
         <v>5.0</v>
       </c>
-      <c r="B78" s="56">
+      <c r="B78" s="121">
         <v>6.0</v>
       </c>
-      <c r="C78" s="56" t="s">
+      <c r="C78" s="121" t="s">
         <v>481</v>
       </c>
-      <c r="D78" s="61" t="s">
+      <c r="D78" s="117" t="s">
         <v>482</v>
       </c>
       <c r="E78" s="121"/>
@@ -14270,16 +14270,16 @@
       <c r="G78" s="121"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
-      <c r="A79" s="55">
+      <c r="A79" s="116">
         <v>6.0</v>
       </c>
-      <c r="B79" s="56">
+      <c r="B79" s="121">
         <v>3.6</v>
       </c>
-      <c r="C79" s="56" t="s">
+      <c r="C79" s="121" t="s">
         <v>475</v>
       </c>
-      <c r="D79" s="61" t="s">
+      <c r="D79" s="117" t="s">
         <v>483</v>
       </c>
       <c r="E79" s="121"/>
@@ -14287,16 +14287,16 @@
       <c r="G79" s="121"/>
     </row>
     <row r="80" ht="14.25" customHeight="1">
-      <c r="A80" s="55">
+      <c r="A80" s="116">
         <v>7.0</v>
       </c>
-      <c r="B80" s="56">
+      <c r="B80" s="121">
         <v>4.0</v>
       </c>
-      <c r="C80" s="56" t="s">
+      <c r="C80" s="121" t="s">
         <v>475</v>
       </c>
-      <c r="D80" s="61" t="s">
+      <c r="D80" s="117" t="s">
         <v>484</v>
       </c>
       <c r="E80" s="121"/>
@@ -14304,16 +14304,16 @@
       <c r="G80" s="121"/>
     </row>
     <row r="81" ht="14.25" customHeight="1">
-      <c r="A81" s="55">
+      <c r="A81" s="116">
         <v>8.0</v>
       </c>
-      <c r="B81" s="56">
+      <c r="B81" s="121">
         <v>1.0</v>
       </c>
-      <c r="C81" s="56" t="s">
+      <c r="C81" s="121" t="s">
         <v>475</v>
       </c>
-      <c r="D81" s="61" t="s">
+      <c r="D81" s="117" t="s">
         <v>485</v>
       </c>
       <c r="E81" s="121"/>
@@ -14321,16 +14321,16 @@
       <c r="G81" s="121"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
-      <c r="A82" s="55">
+      <c r="A82" s="116">
         <v>9.0</v>
       </c>
-      <c r="B82" s="56">
+      <c r="B82" s="121">
         <v>13.0</v>
       </c>
-      <c r="C82" s="56" t="s">
+      <c r="C82" s="121" t="s">
         <v>481</v>
       </c>
-      <c r="D82" s="61" t="s">
+      <c r="D82" s="117" t="s">
         <v>486</v>
       </c>
       <c r="E82" s="121"/>
@@ -14338,19 +14338,19 @@
       <c r="G82" s="121"/>
     </row>
     <row r="83" ht="14.25" customHeight="1">
-      <c r="A83" s="55"/>
-      <c r="B83" s="56"/>
-      <c r="C83" s="56"/>
-      <c r="D83" s="63"/>
+      <c r="A83" s="116"/>
+      <c r="B83" s="121"/>
+      <c r="C83" s="121"/>
+      <c r="D83" s="117"/>
       <c r="E83" s="121"/>
       <c r="F83" s="121"/>
       <c r="G83" s="121"/>
     </row>
     <row r="84" ht="14.25" customHeight="1">
-      <c r="A84" s="55"/>
-      <c r="B84" s="56"/>
-      <c r="C84" s="56"/>
-      <c r="D84" s="61" t="s">
+      <c r="A84" s="116"/>
+      <c r="B84" s="121"/>
+      <c r="C84" s="121"/>
+      <c r="D84" s="117" t="s">
         <v>6</v>
       </c>
       <c r="E84" s="121"/>
@@ -14358,16 +14358,16 @@
       <c r="G84" s="121"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
-      <c r="A85" s="55">
+      <c r="A85" s="116">
         <v>10.0</v>
       </c>
-      <c r="B85" s="56">
+      <c r="B85" s="121">
         <v>20.0</v>
       </c>
-      <c r="C85" s="56" t="s">
+      <c r="C85" s="121" t="s">
         <v>481</v>
       </c>
-      <c r="D85" s="61" t="s">
+      <c r="D85" s="117" t="s">
         <v>487</v>
       </c>
       <c r="E85" s="121"/>
@@ -14375,19 +14375,19 @@
       <c r="G85" s="121"/>
     </row>
     <row r="86" ht="14.25" customHeight="1">
-      <c r="A86" s="55"/>
-      <c r="B86" s="56"/>
-      <c r="C86" s="56"/>
-      <c r="D86" s="63"/>
+      <c r="A86" s="116"/>
+      <c r="B86" s="121"/>
+      <c r="C86" s="121"/>
+      <c r="D86" s="117"/>
       <c r="E86" s="121"/>
       <c r="F86" s="121"/>
       <c r="G86" s="121"/>
     </row>
     <row r="87" ht="14.25" customHeight="1">
-      <c r="A87" s="55"/>
-      <c r="B87" s="56"/>
-      <c r="C87" s="56"/>
-      <c r="D87" s="61" t="s">
+      <c r="A87" s="116"/>
+      <c r="B87" s="121"/>
+      <c r="C87" s="121"/>
+      <c r="D87" s="117" t="s">
         <v>38</v>
       </c>
       <c r="E87" s="121"/>
@@ -14395,16 +14395,16 @@
       <c r="G87" s="121"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
-      <c r="A88" s="55">
+      <c r="A88" s="116">
         <v>11.0</v>
       </c>
-      <c r="B88" s="56">
+      <c r="B88" s="121">
         <v>10.0</v>
       </c>
-      <c r="C88" s="56" t="s">
+      <c r="C88" s="121" t="s">
         <v>488</v>
       </c>
-      <c r="D88" s="61" t="s">
+      <c r="D88" s="117" t="s">
         <v>489</v>
       </c>
       <c r="E88" s="121"/>
@@ -14412,16 +14412,16 @@
       <c r="G88" s="121"/>
     </row>
     <row r="89" ht="14.25" customHeight="1">
-      <c r="A89" s="55">
+      <c r="A89" s="116">
         <v>12.0</v>
       </c>
-      <c r="B89" s="56">
+      <c r="B89" s="121">
         <v>23.0</v>
       </c>
-      <c r="C89" s="56" t="s">
+      <c r="C89" s="121" t="s">
         <v>481</v>
       </c>
-      <c r="D89" s="61" t="s">
+      <c r="D89" s="117" t="s">
         <v>490</v>
       </c>
       <c r="E89" s="121"/>
@@ -14429,16 +14429,16 @@
       <c r="G89" s="121"/>
     </row>
     <row r="90" ht="14.25" customHeight="1">
-      <c r="A90" s="55">
+      <c r="A90" s="116">
         <v>13.0</v>
       </c>
-      <c r="B90" s="56">
+      <c r="B90" s="121">
         <v>7.0</v>
       </c>
-      <c r="C90" s="56" t="s">
+      <c r="C90" s="121" t="s">
         <v>481</v>
       </c>
-      <c r="D90" s="61" t="s">
+      <c r="D90" s="117" t="s">
         <v>491</v>
       </c>
       <c r="E90" s="121"/>
@@ -14754,14 +14754,12 @@
       <c r="G122" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="61">
+  <mergeCells count="57">
     <mergeCell ref="A63:G63"/>
     <mergeCell ref="A64:G64"/>
     <mergeCell ref="B65:D65"/>
     <mergeCell ref="B66:G67"/>
     <mergeCell ref="B70:F70"/>
-    <mergeCell ref="A71:A72"/>
-    <mergeCell ref="B71:B72"/>
     <mergeCell ref="A102:A103"/>
     <mergeCell ref="B102:G103"/>
     <mergeCell ref="B105:G105"/>
@@ -14769,8 +14767,6 @@
     <mergeCell ref="C113:D113"/>
     <mergeCell ref="C119:D119"/>
     <mergeCell ref="C120:D120"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="D71:D72"/>
     <mergeCell ref="B92:G92"/>
     <mergeCell ref="B94:G94"/>
     <mergeCell ref="B96:G96"/>

</xml_diff>

<commit_message>
SPPBJ KAK: merge D:G tiap point + nomor di kolom C
- Template: tambah mergeCell D{r}:G{r} rows 71-76 (teks point satu sel lebar)
- Nomor "1." pindah ke kolom C (indent, sebelum teks merged)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/sppbj/sppbj.xlsx
+++ b/templates/sppbj/sppbj.xlsx
@@ -14154,7 +14154,7 @@
       <c r="B71" s="121" t="s">
         <v>469</v>
       </c>
-      <c r="C71" s="121" t="s">
+      <c r="C71" s="116" t="s">
         <v>470</v>
       </c>
       <c r="D71" s="117" t="s">
@@ -14167,7 +14167,7 @@
     <row r="72">
       <c r="A72" s="116"/>
       <c r="B72" s="121"/>
-      <c r="C72" s="121"/>
+      <c r="C72" s="116"/>
       <c r="D72" s="117"/>
       <c r="E72" s="121"/>
       <c r="F72" s="121"/>
@@ -14176,7 +14176,7 @@
     <row r="73">
       <c r="A73" s="116"/>
       <c r="B73" s="121"/>
-      <c r="C73" s="121"/>
+      <c r="C73" s="116"/>
       <c r="D73" s="117" t="s">
         <v>58</v>
       </c>
@@ -14191,7 +14191,7 @@
       <c r="B74" s="121">
         <v>1.0</v>
       </c>
-      <c r="C74" s="121" t="s">
+      <c r="C74" s="116" t="s">
         <v>475</v>
       </c>
       <c r="D74" s="117" t="s">
@@ -14208,7 +14208,7 @@
       <c r="B75" s="121">
         <v>7.0</v>
       </c>
-      <c r="C75" s="121" t="s">
+      <c r="C75" s="116" t="s">
         <v>477</v>
       </c>
       <c r="D75" s="117" t="s">
@@ -14225,7 +14225,7 @@
       <c r="B76" s="121">
         <v>18.0</v>
       </c>
-      <c r="C76" s="121" t="s">
+      <c r="C76" s="116" t="s">
         <v>475</v>
       </c>
       <c r="D76" s="117" t="s">
@@ -14754,7 +14754,7 @@
       <c r="G122" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="57">
+  <mergeCells count="63">
     <mergeCell ref="A63:G63"/>
     <mergeCell ref="A64:G64"/>
     <mergeCell ref="B65:D65"/>
@@ -14812,6 +14812,12 @@
     <mergeCell ref="E53:G53"/>
     <mergeCell ref="A55:G55"/>
     <mergeCell ref="A62:G62"/>
+    <mergeCell ref="D71:G71"/>
+    <mergeCell ref="D72:G72"/>
+    <mergeCell ref="D73:G73"/>
+    <mergeCell ref="D74:G74"/>
+    <mergeCell ref="D75:G75"/>
+    <mergeCell ref="D76:G76"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins bottom="0.1968503937007874" footer="0.0" header="0.0" left="0.1968503937007874" right="0.1968503937007874" top="0.3937007874015748"/>

</xml_diff>